<commit_message>
fix: deploy workflow for GitHub Pages & update display hardware topology to i3-6100 iGPU
</commit_message>
<xml_diff>
--- a/public/data/benchmarks/gpu_memory_summary.xlsx
+++ b/public/data/benchmarks/gpu_memory_summary.xlsx
@@ -437,7 +437,7 @@
         <v>Intel HD Graphics 530</v>
       </c>
       <c r="C2" t="str">
-        <v>Display &amp; Host Offload iGPU</v>
+        <v>Host Physical Display &amp; Desktop GUI iGPU</v>
       </c>
       <c r="D2" t="str">
         <v>Skylake GT2</v>
@@ -466,7 +466,7 @@
         <v>NVIDIA GeForce GTX 1070</v>
       </c>
       <c r="C3" t="str">
-        <v>Primary Discrete / Display / Head Layer</v>
+        <v>Dedicated AI Compute Node (Pascal GP104)</v>
       </c>
       <c r="D3" t="str">
         <v>Pascal GP104</v>
@@ -478,7 +478,7 @@
         <v>8192</v>
       </c>
       <c r="G3">
-        <v>7980</v>
+        <v>8110</v>
       </c>
       <c r="H3">
         <v>12.8</v>
@@ -613,10 +613,10 @@
         <v>Idle (Docker Ollama Daemon)</v>
       </c>
       <c r="B2">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="C2">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="D2">
         <v>60</v>

</xml_diff>